<commit_message>
Adding files to repo
</commit_message>
<xml_diff>
--- a/4_Day4_HMMs/Data/WolfCollars_JAS.xlsx
+++ b/4_Day4_HMMs/Data/WolfCollars_JAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Jared\GitHub\Courses\China_2026\4_Day4_HMMs\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{379643CF-7782-4561-BF6F-CB7A40802A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED1EEA4-7643-4A17-B90A-F9CBA546B9AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39960" yWindow="540" windowWidth="27075" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SCBI" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="66">
   <si>
     <t>Drop-Off</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t>Vertex Lite</t>
+  </si>
+  <si>
+    <t>Activity Data Download - Currently on laptop</t>
   </si>
 </sst>
 </file>
@@ -1401,8 +1404,8 @@
       <c r="B7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>61</v>
+      <c r="C7" s="27" t="s">
+        <v>65</v>
       </c>
       <c r="D7" s="13">
         <v>32883</v>

</xml_diff>